<commit_message>
feat: add food category selector to UI and implement persistent billing, payment, and analytics data tracking
</commit_message>
<xml_diff>
--- a/docs/test_plan.xlsx
+++ b/docs/test_plan.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="128">
   <si>
     <t xml:space="preserve">Test Case</t>
   </si>
@@ -314,6 +314,9 @@
   </si>
   <si>
     <t xml:space="preserve">Bill total is generated in Billing tab.</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
   <si>
     <t xml:space="preserve">Go to Payments tab and select the bill.</t>
@@ -1799,7 +1802,9 @@
       <c r="D68" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="E68" s="5"/>
+      <c r="E68" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F68" s="5"/>
     </row>
     <row r="69">
@@ -1808,12 +1813,14 @@
         <v>2</v>
       </c>
       <c r="C69" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E69" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D69" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="E69" s="5"/>
       <c r="F69" s="5"/>
     </row>
     <row r="70">
@@ -1822,12 +1829,14 @@
         <v>3</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D70" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="E70" s="5"/>
+        <v>103</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F70" s="5"/>
     </row>
     <row r="71">
@@ -1836,12 +1845,14 @@
         <v>4</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="E71" s="5"/>
+        <v>105</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F71" s="5"/>
     </row>
     <row r="72">
@@ -1850,12 +1861,14 @@
         <v>5</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D72" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="E72" s="5"/>
+        <v>107</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F72" s="5"/>
     </row>
     <row r="73">
@@ -1864,12 +1877,14 @@
         <v>6</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="E73" s="5"/>
+        <v>108</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F73" s="5"/>
     </row>
     <row r="74" ht="27">
@@ -1878,12 +1893,14 @@
         <v>7</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D74" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="E74" s="5"/>
+        <v>110</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F74" s="5"/>
     </row>
     <row r="75" ht="27">
@@ -1892,12 +1909,14 @@
         <v>8</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E75" s="5"/>
+        <v>112</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F75" s="5"/>
     </row>
     <row r="76">
@@ -1906,17 +1925,19 @@
         <v>9</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D76" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="E76" s="5"/>
+        <v>114</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F76" s="5"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B79" s="8"/>
       <c r="C79" s="8"/>
@@ -1930,12 +1951,14 @@
         <v>1</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D80" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="E80" s="5"/>
+        <v>117</v>
+      </c>
+      <c r="E80" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F80" s="5"/>
     </row>
     <row r="81" ht="27">
@@ -1944,12 +1967,14 @@
         <v>2</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="E81" s="5"/>
+        <v>119</v>
+      </c>
+      <c r="E81" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F81" s="5"/>
     </row>
     <row r="82">
@@ -1958,12 +1983,14 @@
         <v>3</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D82" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="E82" s="5"/>
+        <v>121</v>
+      </c>
+      <c r="E82" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F82" s="5"/>
     </row>
     <row r="83" ht="27">
@@ -1972,12 +1999,14 @@
         <v>4</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D83" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="E83" s="5"/>
+        <v>123</v>
+      </c>
+      <c r="E83" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F83" s="5"/>
     </row>
     <row r="84">
@@ -1986,12 +2015,14 @@
         <v>5</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D84" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="E84" s="5"/>
+        <v>125</v>
+      </c>
+      <c r="E84" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F84" s="5"/>
     </row>
     <row r="85">
@@ -2000,12 +2031,14 @@
         <v>6</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D85" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="E85" s="5"/>
+        <v>127</v>
+      </c>
+      <c r="E85" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="F85" s="5"/>
     </row>
   </sheetData>
@@ -2025,13 +2058,13 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2" disablePrompts="0">
-        <x14:dataValidation xr:uid="{74BE66B0-8EC7-46C5-8F6C-CD6A6C88DFB5}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{0FD3DBFB-9614-4BA3-B377-707D61A562B7}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Yes,No"</xm:f>
           </x14:formula1>
           <xm:sqref>E3:E10 E14:E21 E25:E31 E35:E38 E42:E45 E49:E55 E59:E64 E68:E76 E80:E85</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{DF0AB47C-76BD-4522-A0A6-9BF68276A619}" type="list" allowBlank="1" error="Your entry is not in the list (Yes/No)" errorStyle="stop" errorTitle="Invalid Entry" imeMode="noControl" operator="between" prompt="Please select Yes or No" promptTitle="Passed?" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{3EF126B3-DAA8-406A-A146-0F123AC52834}" type="list" allowBlank="1" error="Your entry is not in the list (Yes/No)" errorStyle="stop" errorTitle="Invalid Entry" imeMode="noControl" operator="between" prompt="Please select Yes or No" promptTitle="Passed?" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"Yes,No"</xm:f>
           </x14:formula1>

</xml_diff>